<commit_message>
Anlagenverzeichnis und Aufschlüsselung der Abschreibungen einbinden
Neues Eingabeblatt Anlagen: je Anlage Buchwert und AfA je Prognosejahr,
zugeordnet über die ObjektID. Quellen sind der DATEV-Export
„Inventarübersicht“ (--inventar, KOST1 = Kostenstelle) und die neue
Aufschlüsselung „Buchwert, JE“ / „Abschreibungen JW“ unter der BWA der
Kostenstellenblätter, falls das Verzeichnis die Kostenstelle nicht abdeckt.

- Objekte: AK Gebäude, AK G+B, Kaufjahr, AfA-Satz, Restbuchwert und AfA je
  Jahr kommen aus dem Blatt Anlagen (grün, keine Annahme), sonst wie bisher
- Prognose: neue Spalte AfA bei Halten, Summe der AfA je Anlage; jede Anlage
  läuft für sich aus
- BWA-Blätter je Kostenstelle mit Aufschlüsselung je Anlage und Jahr
- Prüfung: Hinweise auf Anlagen ohne Objekt und auf Abweichung zu BWA 1240
- Vorlagen, Prüfskripte, README und Projektplan Abschnitt 21

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HKaJyLE1UDFHJLz1dAoyYw
</commit_message>
<xml_diff>
--- a/vorlagen/Kostenstellen_BWA_Vorlage.xlsx
+++ b/vorlagen/Kostenstellen_BWA_Vorlage.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Alle Objekte" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="KSt 1" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="KSt 2" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Alle Objekte" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KSt 1" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KSt 2" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3171,7 +3171,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:AN50"/>
+  <dimension ref="B2:AN61"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="3" max="3"/>
@@ -5781,6 +5781,71 @@
       <c r="AM50" s="4" t="n"/>
       <c r="AN50" s="4" t="n"/>
     </row>
+    <row r="53">
+      <c r="C53" s="1" t="inlineStr">
+        <is>
+          <t>Buchwert, JE</t>
+        </is>
+      </c>
+      <c r="G53" t="n">
+        <v>496000</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Wohnbau 1</t>
+        </is>
+      </c>
+      <c r="G54" t="n">
+        <v>496000</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="C56" s="1" t="inlineStr">
+        <is>
+          <t>Abschreibungen JW</t>
+        </is>
+      </c>
+      <c r="G56" t="n">
+        <v>16000</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="G57" t="n">
+        <v>16000</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>Wohnbau 1</t>
+        </is>
+      </c>
+      <c r="G58" t="n">
+        <v>16000</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="C60" s="1" t="inlineStr">
+        <is>
+          <t>Abschreibungen MW</t>
+        </is>
+      </c>
+      <c r="G60" t="n">
+        <v>1333.333333333333</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Wohnbau 1</t>
+        </is>
+      </c>
+      <c r="G61" t="n">
+        <v>1333.33</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5792,7 +5857,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:AN50"/>
+  <dimension ref="B2:AN70"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="3" max="3"/>
@@ -8522,6 +8587,158 @@
       <c r="AM50" s="4" t="n"/>
       <c r="AN50" s="4" t="n"/>
     </row>
+    <row r="53">
+      <c r="C53" s="1" t="inlineStr">
+        <is>
+          <t>Buchwert, JE</t>
+        </is>
+      </c>
+      <c r="G53" t="n">
+        <v>941000</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>Wohnbau 7</t>
+        </is>
+      </c>
+      <c r="G54" t="n">
+        <v>876000</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>Außenanlagen 7</t>
+        </is>
+      </c>
+      <c r="G55" t="n">
+        <v>15000</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>Anbau im Bau</t>
+        </is>
+      </c>
+      <c r="G56" t="n">
+        <v>50000</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>sonstige</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="C59" s="1" t="inlineStr">
+        <is>
+          <t>Abschreibungen JW</t>
+        </is>
+      </c>
+      <c r="G59" t="n">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="G60" t="n">
+        <v>30000</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Wohnbau</t>
+        </is>
+      </c>
+      <c r="G61" t="n">
+        <v>24000</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Außenanlagen</t>
+        </is>
+      </c>
+      <c r="G62" t="n">
+        <v>6000</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>Anbau im Bau</t>
+        </is>
+      </c>
+      <c r="G63" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>sonstige</t>
+        </is>
+      </c>
+      <c r="G64" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="C66" s="1" t="inlineStr">
+        <is>
+          <t>Abschreibungen MW</t>
+        </is>
+      </c>
+      <c r="G66" t="n">
+        <v>2500</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>Wohnbau</t>
+        </is>
+      </c>
+      <c r="G67" t="n">
+        <v>2000</v>
+      </c>
+    </row>
+    <row r="68">
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>Außenanlagen</t>
+        </is>
+      </c>
+      <c r="G68" t="n">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="69">
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>Anbau im Bau</t>
+        </is>
+      </c>
+      <c r="G69" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="70">
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>sonstige</t>
+        </is>
+      </c>
+      <c r="G70" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>